<commit_message>
Add verified trace memory for scalable conversation context and regeneration safeguards
</commit_message>
<xml_diff>
--- a/pipeclaw/backend/generated_teacher_traces/task1_deliverables/teacher_trace_statistics.xlsx
+++ b/pipeclaw/backend/generated_teacher_traces/task1_deliverables/teacher_trace_statistics.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset Sources" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Types" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Types" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constraint Types" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constraint Outcomes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Outcomes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Levels" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intervention Labels" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk x Intervention" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Split Statistics" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Statistics" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Statistics" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method Notes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dataset Sources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Scenario Types" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Task Types" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Constraint Types" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Constraint Outcomes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Rule Outcomes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Risk Levels" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Intervention Labels" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Risk x Intervention" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Split Statistics" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Evidence Statistics" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Quality Statistics" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Method Notes" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dataset Sources'!$1:$1</definedName>
@@ -46,7 +46,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,12 +86,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="007F6000"/>
       <sz val="10"/>
     </font>
@@ -114,7 +108,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -149,11 +143,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -204,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -230,13 +219,10 @@
     <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -245,13 +231,13 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -331,14 +317,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -362,10 +348,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
@@ -396,8 +382,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -423,8 +409,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -450,14 +436,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -481,10 +467,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
@@ -515,8 +501,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -542,8 +528,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -569,14 +555,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -600,10 +586,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
@@ -634,8 +620,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -661,8 +647,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -688,14 +674,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -719,10 +705,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
@@ -753,8 +739,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -780,8 +766,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -807,14 +793,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -837,10 +823,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
@@ -849,12 +835,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Risk Levels'!$A$2:$A$6</f>
+              <f>'Risk Levels'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Risk Levels'!$B$2:$B$6</f>
+              <f>'Risk Levels'!$B$2:$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -871,7 +857,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -886,9 +872,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -898,7 +884,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -913,9 +899,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -925,7 +911,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -940,9 +926,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -952,7 +938,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -967,9 +953,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -979,7 +965,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -994,9 +980,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1157,8 +1143,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditTable08" displayName="AuditTable08" ref="A1:C6" headerRowCount="1">
-  <autoFilter ref="A1:C6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AuditTable08" displayName="AuditTable08" ref="A1:C5" headerRowCount="1">
+  <autoFilter ref="A1:C5"/>
   <tableColumns count="3">
     <tableColumn id="1" name="risk_level"/>
     <tableColumn id="2" name="count"/>
@@ -1181,8 +1167,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AuditTable10" displayName="AuditTable10" ref="A1:F6" headerRowCount="1">
-  <autoFilter ref="A1:F6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AuditTable10" displayName="AuditTable10" ref="A1:F5" headerRowCount="1">
+  <autoFilter ref="A1:F5"/>
   <tableColumns count="6">
     <tableColumn id="1" name="risk_level"/>
     <tableColumn id="2" name="monitoring_only"/>
@@ -1508,7 +1494,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-07-24T15:00:46.557723+00:00</t>
+          <t>2026-07-28T10:45:42.533796+00:00</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1557,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>806</v>
+        <v>823</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1581,7 +1567,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.7070175438596491</v>
+        <v>0.7219298245614035</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -1591,7 +1577,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.951754</v>
+        <v>0.869298</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1600,8 +1586,8 @@
           <t>Task 1 quality pass rate</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
-        <v>0.887719</v>
+      <c r="B11" s="8" t="n">
+        <v>0.857895</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -1611,7 +1597,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>6.408771929824561</v>
+        <v>7.63421052631579</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1631,7 +1617,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>153.5140350877193</v>
+        <v>155.4921052631579</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1641,7 +1627,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>0.6043859649122807</v>
+        <v>0.6096491228070176</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1651,7 +1637,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
@@ -1661,7 +1647,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1688,7 +1674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1700,145 +1686,123 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>monitoring_only</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>no_intervention</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>not_applicable</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>operator_attention_required</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>row_total</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="F2" s="12" t="n">
-        <v>13</v>
+      <c r="B2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="12" t="n">
-        <v>36</v>
-      </c>
-      <c r="D3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>36</v>
+      <c r="B3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>38</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>97</v>
+      <c r="B4" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>not_applicable</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>992</v>
-      </c>
-      <c r="E5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>992</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>2</v>
+      <c r="B5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>1001</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>1001</v>
       </c>
     </row>
   </sheetData>
@@ -1881,157 +1845,157 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>split</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>master_samples</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>scenario_count</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>session_count</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>quality_pass</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>sft_eligible</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>sft_eligible_rate</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>average_evidence_items</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>average_answer_chars</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>train</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B2" s="11" t="n">
         <v>902</v>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="11" t="n">
         <v>64</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="11" t="n">
         <v>224</v>
       </c>
-      <c r="E2" s="12" t="n">
-        <v>797</v>
-      </c>
-      <c r="F2" s="12" t="n">
+      <c r="E2" s="11" t="n">
+        <v>759</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>612</v>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>0.6784922394678492</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>7.585365853658536</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>153.069844789357</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>124</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>113</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="G3" s="11" t="n">
         <v>105</v>
       </c>
-      <c r="G2" s="12" t="n">
-        <v>611</v>
-      </c>
-      <c r="H2" s="13" t="n">
-        <v>0.6773835920177383</v>
-      </c>
-      <c r="I2" s="12" t="n">
-        <v>6.390243902439025</v>
-      </c>
-      <c r="J2" s="12" t="n">
-        <v>151.8414634146341</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>valid</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="n">
-        <v>124</v>
-      </c>
-      <c r="C3" s="12" t="n">
+      <c r="H3" s="12" t="n">
+        <v>0.8467741935483871</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>7.814516129032258</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>165.5725806451613</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>114</v>
+      </c>
+      <c r="C4" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D4" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="E3" s="12" t="n">
-        <v>110</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>14</v>
-      </c>
-      <c r="G3" s="12" t="n">
-        <v>107</v>
-      </c>
-      <c r="H3" s="13" t="n">
-        <v>0.8629032258064516</v>
-      </c>
-      <c r="I3" s="12" t="n">
-        <v>6.419354838709677</v>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>166.0322580645161</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="n">
-        <v>114</v>
-      </c>
-      <c r="C4" s="12" t="n">
+      <c r="E4" s="11" t="n">
+        <v>106</v>
+      </c>
+      <c r="F4" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D4" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>105</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>88</v>
-      </c>
-      <c r="H4" s="13" t="n">
-        <v>0.7719298245614035</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>6.543859649122807</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>153.1315789473684</v>
+      <c r="G4" s="11" t="n">
+        <v>106</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>0.9298245614035088</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>7.824561403508772</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>163.6929824561404</v>
       </c>
     </row>
   </sheetData>
@@ -2080,7 +2044,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -2088,232 +2052,232 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>dataset_source</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>scenario_type</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>zero_evidence_samples</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>minimum</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>p25</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>median</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>p75</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>p90</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>p95</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>maximum</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Pipeline_Full_Life_Cycle_Test_Dataset-v4</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>openclaw</t>
         </is>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="11" t="n">
         <v>256</v>
       </c>
-      <c r="E2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="12" t="n">
-        <v>3.623333333333334</v>
-      </c>
-      <c r="I2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="12" t="n">
-        <v>13.10000000000002</v>
-      </c>
-      <c r="K2" s="12" t="n">
-        <v>29</v>
-      </c>
-      <c r="L2" s="12" t="n">
-        <v>62</v>
+      <c r="E2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>17.10000000000002</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Pipeline_Full_Life_Cycle_Test_Dataset-v4</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>pipeformer</t>
         </is>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="D3" s="12" t="n">
-        <v>93</v>
-      </c>
-      <c r="E3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="12" t="n">
+      <c r="D3" s="11" t="n">
+        <v>98</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="H3" s="12" t="n">
-        <v>15.56</v>
-      </c>
-      <c r="I3" s="12" t="n">
+      <c r="H3" s="11" t="n">
+        <v>18.255</v>
+      </c>
+      <c r="I3" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="J3" s="12" t="n">
-        <v>43</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>51.24999999999991</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>78</v>
+      <c r="J3" s="11" t="n">
+        <v>54.39999999999998</v>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>169</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Pipeline_Full_Life_Cycle_Test_Dataset-v7</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>pipeformer</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="12" t="n">
+      <c r="D4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="F4" s="12" t="n">
-        <v>20.25</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="H4" s="12" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>52</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>61</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>62.05</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>64</v>
+      <c r="F4" s="11" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>42</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>52.65</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>61.25</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>108</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>112.35</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>179</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>pipeclaw_dataset_v2</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>openclaw</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="11" t="n">
         <v>600</v>
       </c>
-      <c r="D5" s="12" t="n">
-        <v>556</v>
-      </c>
-      <c r="E5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>2.665</v>
-      </c>
-      <c r="I5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>23</v>
-      </c>
-      <c r="L5" s="12" t="n">
+      <c r="D5" s="11" t="n">
+        <v>548</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>2.905</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>29.04999999999995</v>
+      </c>
+      <c r="L5" s="11" t="n">
         <v>103</v>
       </c>
     </row>
@@ -2353,167 +2317,167 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>quality_dimension</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>fail_or_needs_review</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>not_applicable</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>applicable_count</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>applicable_pass_rate</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>schema</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B2" s="11" t="n">
         <v>1140</v>
       </c>
-      <c r="C2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="12" t="n">
+      <c r="C2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11" t="n">
         <v>1140</v>
       </c>
-      <c r="F2" s="13" t="n">
+      <c r="F2" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>numerical_consistency</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>1040</v>
-      </c>
-      <c r="C3" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="12" t="n">
+      <c r="B3" s="11" t="n">
+        <v>1099</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11" t="n">
         <v>1140</v>
       </c>
-      <c r="F3" s="13" t="n">
-        <v>0.9122807017543859</v>
+      <c r="F3" s="12" t="n">
+        <v>0.9640350877192982</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>rule_consistency</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>148</v>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>992</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>148</v>
-      </c>
-      <c r="F4" s="13" t="n">
+      <c r="B4" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>1001</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="F4" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>dispatch_consistency</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>148</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>992</v>
-      </c>
-      <c r="E5" s="12" t="n">
-        <v>148</v>
-      </c>
-      <c r="F5" s="13" t="n">
+      <c r="B5" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>1001</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="F5" s="12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>native_quality</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>1085</v>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>55</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="12" t="n">
+      <c r="B6" s="11" t="n">
+        <v>991</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>149</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11" t="n">
         <v>1140</v>
       </c>
-      <c r="F6" s="13" t="n">
-        <v>0.9517543859649122</v>
+      <c r="F6" s="12" t="n">
+        <v>0.8692982456140351</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>task1_quality</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>1012</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>128</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="12" t="n">
+      <c r="B7" s="11" t="n">
+        <v>978</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>162</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="n">
         <v>1140</v>
       </c>
-      <c r="F7" s="13" t="n">
-        <v>0.887719298245614</v>
+      <c r="F7" s="12" t="n">
+        <v>0.8578947368421053</v>
       </c>
     </row>
   </sheetData>
@@ -2560,120 +2524,120 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>topic</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>definition</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Standalone Task 1.9 data-statistics tables for the master teacher-trace dataset.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>SFT eligible</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Task 1 pass, no explicit SFT exclusion, and all preceding conversation turns pass quality.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Evidence items</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Recursive count of non-empty scalar/list items in the top-level evidence object.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Scenario types</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Scenario-family distribution across all teacher-trace records.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Task types</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>PipeFormer task-subtype distribution across PipeFormer scenario records only; unspecified means no subtype was stored.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Constraint requested</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>A category listed in constraint_check.requested_categories.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Constraint evaluated</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Requested category with pass, warning, or fail in category_status.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Percentiles</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Nearest-rank interpolation over per-record evidence-item counts.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Workbook formulas</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Fixed verification snapshot; no formulas or external links are used.</t>
         </is>
@@ -2713,297 +2677,297 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Pipeline_Full_Life_Cycle_Test_Dataset-v4</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Pipeline_Full_Life_Cycle_Test_Dataset-v7</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>pipeclaw_dataset_v2</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B2" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="11" t="n">
         <v>600</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="12" t="n">
         <v>0.4385964912280702</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="12" t="n">
         <v>0.03508771929824561</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="12" t="n">
         <v>0.5263157894736842</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>scenario_count</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="11" t="n">
         <v>70</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="11" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>session_count</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="11" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>openclaw</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="C6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="12" t="n">
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11" t="n">
         <v>600</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>pipeformer</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>train</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="11" t="n">
         <v>390</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="11" t="n">
         <v>480</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>valid</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="11" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="11" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>quality_pass</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
-        <v>444</v>
-      </c>
-      <c r="C11" s="12" t="n">
-        <v>35</v>
-      </c>
-      <c r="D11" s="12" t="n">
-        <v>533</v>
+      <c r="B11" s="11" t="n">
+        <v>385</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>586</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
-        <v>56</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>67</v>
+      <c r="B12" s="11" t="n">
+        <v>115</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>33</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>quality_pass_rate</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
-        <v>0.888</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>0.8883333333333333</v>
+      <c r="B13" s="12" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>0.9766666666666667</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>average_evidence_items</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
-        <v>8.398</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>2.665</v>
+      <c r="B14" s="11" t="n">
+        <v>9.708</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>52.65</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>2.905</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>median_evidence_items</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="D15" s="12" t="n">
+      <c r="B15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>42</v>
+      </c>
+      <c r="D15" s="11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>p95_evidence_items</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
-        <v>43</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>62.05</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>23</v>
+      <c r="B16" s="11" t="n">
+        <v>50.04999999999995</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>112.35</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>29.04999999999995</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>average_answer_chars</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
-        <v>209.694</v>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>379.775</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>91.61333333333333</v>
+      <c r="B17" s="11" t="n">
+        <v>213.704</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>375.675</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>92.30333333333333</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>average_tool_calls</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
-        <v>0.832</v>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>0.205</v>
+      <c r="B18" s="11" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0.1683333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -3040,45 +3004,45 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>scenario_type</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>openclaw</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B2" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="C2" s="13" t="n">
+      <c r="C2" s="12" t="n">
         <v>0.7894736842105263</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>pipeformer</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="11" t="n">
         <v>240</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="12" t="n">
         <v>0.2105263157894737</v>
       </c>
     </row>
@@ -3128,71 +3092,71 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>pipeformer_task_type</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>prediction</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" s="13" t="n">
-        <v>0.008333333333333333</v>
+      <c r="B2" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>0.01666666666666667</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>prediction_and_verification</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>93</v>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>0.3875</v>
+      <c r="B3" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>0.375</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>unspecified</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>144</v>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>0.6</v>
+      <c r="B4" s="11" t="n">
+        <v>145</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>0.6041666666666666</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>verification</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="12" t="n">
         <v>0.004166666666666667</v>
       </c>
     </row>
@@ -3242,124 +3206,124 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>constraint_type</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>abnormality_warning</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C2" s="13" t="n">
-        <v>0.1241914618369987</v>
+      <c r="B2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>0.1226912928759894</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>compressor</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>0.1254851228978008</v>
+      <c r="B3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>dispatch_priority</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>0.1254851228978008</v>
+      <c r="B4" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>equipment_regulation</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>0.1241914618369987</v>
+      <c r="B5" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>flow</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>0.1241914618369987</v>
+      <c r="B6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>human_intervention</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C7" s="13" t="n">
-        <v>0.1254851228978008</v>
+      <c r="B7" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>linepack</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C8" s="13" t="n">
-        <v>0.1254851228978008</v>
+      <c r="B8" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>pressure</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>0.1254851228978008</v>
+      <c r="B9" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>0.1253298153034301</v>
       </c>
     </row>
   </sheetData>
@@ -3411,330 +3375,330 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>constraint_category</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>requested</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>not_evaluated_or_missing</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>coverage_rate</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>pass_rate</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>non_pass_rate</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>abnormality_warning</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C2" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D2" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="E2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="13" t="n">
+      <c r="B2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="13" t="n">
+      <c r="I2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="13" t="n">
+      <c r="J2" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>compressor</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C3" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D3" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="E3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="13" t="n">
+      <c r="B3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="13" t="n">
+      <c r="I3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="13" t="n">
+      <c r="J3" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>dispatch_priority</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="13" t="n">
+      <c r="B4" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="13" t="n">
+      <c r="I4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="13" t="n">
+      <c r="J4" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>equipment_regulation</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>41</v>
-      </c>
-      <c r="E5" s="12" t="n">
+      <c r="B5" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="E5" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="F5" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="13" t="n">
+      <c r="F5" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="13" t="n">
-        <v>0.4270833333333333</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>0.5729166666666666</v>
+      <c r="I5" s="12" t="n">
+        <v>0.4736842105263158</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>0.5263157894736842</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>flow</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="13" t="n">
+      <c r="B6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>human_intervention</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D7" s="12" t="n">
+      <c r="B7" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D7" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="11" t="n">
+        <v>67</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>0.2947368421052631</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0.7052631578947368</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>linepack</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D8" s="11" t="n">
         <v>69</v>
       </c>
-      <c r="F7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="13" t="n">
+      <c r="E8" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="13" t="n">
-        <v>0.288659793814433</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>0.711340206185567</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>linepack</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>74</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>23</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="13" t="n">
+      <c r="I8" s="12" t="n">
+        <v>0.7263157894736842</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>0.2736842105263158</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="13" t="n">
-        <v>0.7628865979381443</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>0.2371134020618557</v>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>pressure</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="13" t="n">
+      <c r="I9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="13" t="n">
+      <c r="J9" s="12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3808,692 +3772,692 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>rule_id</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>not_evaluated_or_missing</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>pass_rate</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>non_pass_rate</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>abnormal_pressure_drop</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C2" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="13" t="n">
+      <c r="B2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="13" t="n">
+      <c r="H2" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>boundary_control_adjustment_magnitude</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>95</v>
-      </c>
-      <c r="C3" s="12" t="n">
-        <v>40</v>
-      </c>
-      <c r="D3" s="12" t="n">
+      <c r="B3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="D3" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="E3" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="F3" s="12" t="n">
+      <c r="E3" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>0.4736842105263158</v>
+      </c>
+      <c r="H3" s="12" t="n">
+        <v>0.5263157894736842</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>boundary_flow_change_rate</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="13" t="n">
-        <v>0.4210526315789473</v>
-      </c>
-      <c r="H3" s="13" t="n">
-        <v>0.5789473684210527</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>boundary_flow_change_rate</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="13" t="n">
+      <c r="H4" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>compressor_load_limit</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>compressor_load_limit</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="13" t="n">
+      <c r="H5" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>compressor_power_change</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>compressor_power_change</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="13" t="n">
+      <c r="H6" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>compressor_ratio_boundary</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>compressor_ratio_boundary</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="13" t="n">
+      <c r="H7" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>compressor_rotational_speed_limit</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>compressor_rotational_speed_limit</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="13" t="n">
+      <c r="H8" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>dispatch_priority_rules</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>dispatch_priority_rules</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="13" t="n">
+      <c r="H9" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>energy_consumption_cost</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>energy_consumption_cost</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C10" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="13" t="n">
+      <c r="H10" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>equipment_anomaly</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>equipment_anomaly</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C11" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="13" t="n">
+      <c r="H11" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>flow_capacity_check</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>flow_capacity_check</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="13" t="n">
+      <c r="H12" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>flow_ramp_check</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>flow_ramp_check</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="13" t="n">
+      <c r="H13" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>human_intervention_rules</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>67</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>0.2947368421052631</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>0.7052631578947368</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>key_node_pressure_margin</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>human_intervention_rules</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="D14" s="12" t="n">
+      <c r="H15" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>linepack_change_rate</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>linepack_decline_and_recovery</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C17" s="11" t="n">
         <v>69</v>
       </c>
-      <c r="E14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="13" t="n">
-        <v>0.288659793814433</v>
-      </c>
-      <c r="H14" s="13" t="n">
-        <v>0.711340206185567</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>key_node_pressure_margin</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="13" t="n">
+      <c r="D17" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>0.7263157894736842</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>0.2736842105263158</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>linepack_peak_shaving_reserve</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>linepack_change_rate</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="13" t="n">
+      <c r="H18" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>node_pressure_operating_window</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>linepack_decline_and_recovery</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>74</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>23</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>0.7628865979381443</v>
-      </c>
-      <c r="H17" s="13" t="n">
-        <v>0.2371134020618557</v>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>linepack_peak_shaving_reserve</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="13" t="n">
+      <c r="H19" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>potential_leak_signal</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>node_pressure_operating_window</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="D19" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="13" t="n">
+      <c r="H20" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>pressure_regulator_range</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>potential_leak_signal</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C20" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D20" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="13" t="n">
+      <c r="H21" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>sudden_flow_change</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>pressure_regulator_range</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C21" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="13" t="n">
+      <c r="H22" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>supply_demand_balance</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>sudden_flow_change</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C22" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D22" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="13" t="n">
+      <c r="H23" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>valve_opening_range</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>supply_demand_balance</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C23" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>valve_opening_range</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="C24" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="13" t="n">
+      <c r="H24" s="12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4545,98 +4509,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="C2" s="13" t="n">
-        <v>0.01140350877192983</v>
+      <c r="B2" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>0.007017543859649123</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>36</v>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>0.03157894736842105</v>
+      <c r="B3" s="11" t="n">
+        <v>38</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>97</v>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>0.08508771929824561</v>
+      <c r="B4" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>0.08157894736842106</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>not_applicable</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>992</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>0.8701754385964913</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>0.001754385964912281</v>
+      <c r="B5" s="11" t="n">
+        <v>1001</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>0.8780701754385964</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C6">
+  <conditionalFormatting sqref="C2:C5">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -4681,72 +4632,72 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>intervention_label</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>monitoring_only</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
-        <v>99</v>
-      </c>
-      <c r="C2" s="13" t="n">
-        <v>0.0868421052631579</v>
+      <c r="B2" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>0.08157894736842106</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>no_intervention</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>36</v>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>0.03157894736842105</v>
+      <c r="B3" s="11" t="n">
+        <v>38</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>not_applicable</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>992</v>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>0.8701754385964913</v>
+      <c r="B4" s="11" t="n">
+        <v>1001</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>0.8780701754385964</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>operator_attention_required</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>0.01140350877192983</v>
+      <c r="B5" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>0.007017543859649123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>